<commit_message>
Update points for RCB vs SRH
</commit_message>
<xml_diff>
--- a/detailed_output.xlsx
+++ b/detailed_output.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2740,6 +2740,606 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>HARSH</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>SRH6</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Salil Arora</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>9</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Batting</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>HARSH</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>RCB3</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Devdutt Padikkal</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>61</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Batting</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>SOMIL</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>RCB4</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Rajat Patidar</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>31</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Batting</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>SOMIL</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>RCB6</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Tim David</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>16</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Batting</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>SOMIL</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>RCB_B3</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Abhinandan Singh</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Bowling</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>SOMIL</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>SRH_B4</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Harsh Dubey</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>1</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Bowling</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>RAM</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>SRH3</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Ishan Kishan</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>80</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Batting</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>RAM</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>RCB5</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Jitesh Sharma</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Batting</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>RAM</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>RCB_B1</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Jacob Duffy</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>3</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Bowling</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>RAM</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>RCB_B2</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Bhuvneshwar Kumar</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Bowling</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>AJAY</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>SRH2</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Abhishek Sharma</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>7</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Batting</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>AJAY</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>RCB2</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Virat Kohli</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>69</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Batting</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>AJAY</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>SRH4</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Nitish Kumar Reddy</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Batting</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>AJAY</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>SRH_B2</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Jaydev Unadkat</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>1</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Bowling</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>AJAY</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>RCB_B4</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Romario Shepherd</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>3</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Bowling</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>AJAY</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>SRH_B3</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>David Payne</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>2</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Bowling</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>PANDEY</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>SRH5</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Heinrich Klaasen</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>31</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Batting</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>PANDEY</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>SRH_B1</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Nitish Kumar Reddy</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>0</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Bowling</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>AKASH</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>SRH1</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Travis Head</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>11</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Batting</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>AKASH</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>RCB vs SRH</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>RCB1</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Philip Salt</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>8</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Batting</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>